<commit_message>
Unit test updates and test tracker
</commit_message>
<xml_diff>
--- a/docs/PaymentTestUseCase.xlsx
+++ b/docs/PaymentTestUseCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39C1541-C192-4A62-B768-859D65B401FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B79AB1A-188A-40E1-B541-ADAA3E010C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EFBCE3D8-2899-4030-A5B5-F152C55CBB1D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="163">
   <si>
     <t>Test ID</t>
   </si>
@@ -511,6 +511,9 @@
   </si>
   <si>
     <t>Missing - Google Pay unsupported browser test</t>
+  </si>
+  <si>
+    <t>Completion of Test case</t>
   </si>
 </sst>
 </file>
@@ -862,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFCCBEB0-E0ED-472C-81D6-C3F3F80DAD42}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.5703125" bestFit="1" customWidth="1"/>
@@ -871,9 +874,10 @@
     <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="64.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -895,8 +899,11 @@
       <c r="G1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -919,7 +926,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -942,7 +949,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -965,7 +972,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -988,7 +995,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1011,7 +1018,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1034,7 +1041,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1057,7 +1064,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1080,7 +1087,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1103,7 +1110,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1126,7 +1133,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -1149,7 +1156,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1172,7 +1179,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -1195,7 +1202,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -1218,7 +1225,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>57</v>
       </c>

</xml_diff>